<commit_message>
feat: publish M2 T042 gameplay and clean repository contents
</commit_message>
<xml_diff>
--- a/Shared/config/Defines/__tables__.xlsx
+++ b/Shared/config/Defines/__tables__.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1162,6 +1162,106 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>TbShop</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Shop</t>
+        </is>
+      </c>
+      <c r="D22" t="b">
+        <v>1</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>shop.xlsx</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>商店</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>TbMapInstance</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MapInstance</t>
+        </is>
+      </c>
+      <c r="D23" t="b">
+        <v>1</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>mapinstance.xlsx</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>instanceId</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>map</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>M2固定灰盒地图实例</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>TbPlayerInit</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>PlayerInit</t>
+        </is>
+      </c>
+      <c r="D24" t="b">
+        <v>1</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>playerinit.xlsx</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>one</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>玩法初始化（货币仍取 Global/player 默认）</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>